<commit_message>
Added ProjectPlan.xlsx and updated Inventory
Added ProjectPlan.xlsx and updated Inventory
</commit_message>
<xml_diff>
--- a/Inventory.xlsx
+++ b/Inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Lakshman\Bits related docs\gits\PMO-Office\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CC37789-1FAB-4C9A-B746-4B68C47766E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098D72BD-D6A8-4F9E-92AE-44C036481FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5674" yWindow="600" windowWidth="24686" windowHeight="13260" xr2:uid="{0EF1E5E7-D8B3-44C8-AF76-218B17634589}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Item</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>hyderabad</t>
+  </si>
+  <si>
+    <t>Wireless Mouse</t>
+  </si>
+  <si>
+    <t>Coimbatore</t>
   </si>
 </sst>
 </file>
@@ -433,8 +439,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAEDEC9-1BC9-4680-A108-5CD1072C0401}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="13.921875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
@@ -467,6 +476,17 @@
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>